<commit_message>
feat: Update equipment and marble configurations for enhanced gameplay mechanics
Modified equipment and marble configuration files to improve gameplay dynamics. Adjusted cooldown values for swords and increased speed attributes for marbles, enhancing their performance. Added new prefab files for equipment and marbles, along with associated metadata, to support the updated gameplay features. Introduced a new scene for testing combat mechanics, along with a combat manager to facilitate battle logic.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -1489,7 +1489,7 @@
         <v>1</v>
       </c>
       <c r="K5" s="30">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="L5" s="29"/>
       <c r="M5" s="31"/>
@@ -1518,7 +1518,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="30">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="L6" s="29"/>
       <c r="M6" s="31"/>

</xml_diff>

<commit_message>
feat: Enhance equipment and marble configurations with new abilities and structural updates
Updated the equipment and marble configuration files to introduce new abilities such as ArmorAbsorbDamageAbility and SwordCollisionAttackAbility. Restructured XML and JSON files for improved gameplay dynamics, ensuring better integration with the combat system. Added new ability interfaces and refined the registration process for a more modular approach to gameplay mechanics. Removed obsolete files and improved organization across the configuration structure.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
   <si>
     <t>##var</t>
   </si>
@@ -94,7 +94,7 @@
     <t>string</t>
   </si>
   <si>
-    <t>list,string</t>
+    <t>list,EquipmentAbilityConfig</t>
   </si>
   <si>
     <t>int?</t>
@@ -121,13 +121,16 @@
     <t>sword</t>
   </si>
   <si>
-    <t>0</t>
-  </si>
-  <si>
     <t>剑</t>
   </si>
   <si>
-    <t>1</t>
+    <t>shield</t>
+  </si>
+  <si>
+    <t>盾</t>
+  </si>
+  <si>
+    <t>armor_absorb_damage,0</t>
   </si>
 </sst>
 </file>
@@ -520,28 +523,10 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="13">
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
       <top/>
       <bottom/>
       <diagonal/>
@@ -596,43 +581,6 @@
       <right style="medium">
         <color auto="1"/>
       </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color auto="1"/>
       </top>
@@ -765,7 +713,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="10">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="5">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
@@ -777,34 +725,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="13">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="14">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="13">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="15">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="16">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
@@ -889,18 +837,30 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -908,82 +868,79 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1297,235 +1254,274 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q6"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="5"/>
+  <dimension ref="A1:Q8"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="7"/>
   <cols>
-    <col min="2" max="2" width="11.5454545454545" customWidth="1"/>
-    <col min="6" max="6" width="14" customWidth="1"/>
-    <col min="7" max="7" width="9" style="1"/>
-    <col min="8" max="8" width="9" style="2"/>
-    <col min="9" max="9" width="8.09090909090909" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.2727272727273" customWidth="1"/>
-    <col min="11" max="11" width="10.3636363636364" style="2" customWidth="1"/>
-    <col min="12" max="12" width="15.2727272727273" style="1" customWidth="1"/>
-    <col min="13" max="13" width="18.3636363636364" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="17.7272727272727" customWidth="1"/>
-    <col min="16" max="16" width="20.1818181818182" customWidth="1"/>
-    <col min="17" max="17" width="11.5454545454545" style="2" customWidth="1"/>
+    <col min="1" max="1" width="9" style="1"/>
+    <col min="2" max="2" width="11.5454545454545" style="1" customWidth="1"/>
+    <col min="3" max="5" width="9" style="1"/>
+    <col min="6" max="6" width="33.6363636363636" style="2" customWidth="1"/>
+    <col min="7" max="7" width="9" style="3"/>
+    <col min="8" max="8" width="9" style="4"/>
+    <col min="9" max="9" width="8.09090909090909" style="3" customWidth="1"/>
+    <col min="10" max="10" width="26.2727272727273" style="1" customWidth="1"/>
+    <col min="11" max="11" width="10.3636363636364" style="4" customWidth="1"/>
+    <col min="12" max="12" width="15.2727272727273" style="3" customWidth="1"/>
+    <col min="13" max="13" width="18.3636363636364" style="1" customWidth="1"/>
+    <col min="14" max="14" width="14" style="1" customWidth="1"/>
+    <col min="15" max="15" width="17.7272727272727" style="1" customWidth="1"/>
+    <col min="16" max="16" width="20.1818181818182" style="1" customWidth="1"/>
+    <col min="17" max="17" width="11.5454545454545" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="7"/>
-      <c r="I1" s="6"/>
-      <c r="J1" s="4"/>
-      <c r="K1" s="7"/>
-      <c r="L1" s="6"/>
-      <c r="M1" s="4"/>
-      <c r="N1" s="4"/>
-      <c r="O1" s="4"/>
-      <c r="P1" s="4"/>
-      <c r="Q1" s="7"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="9"/>
     </row>
     <row r="2" spans="1:17">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="9" t="s">
+      <c r="F2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="10" t="s">
+      <c r="G2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="11" t="s">
+      <c r="H2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="10" t="s">
+      <c r="I2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="8" t="s">
+      <c r="J2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="11" t="s">
+      <c r="K2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="10" t="s">
+      <c r="L2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="8" t="s">
+      <c r="M2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="N2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="O2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="P2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="11" t="s">
+      <c r="Q2" s="13" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:17">
-      <c r="A3" s="12" t="s">
+      <c r="A3" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="13" t="s">
+      <c r="B3" s="14"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="14" t="s">
+      <c r="E3" s="16" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="15" t="s">
+      <c r="F3" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="17" t="s">
+      <c r="H3" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="I3" s="16" t="s">
+      <c r="I3" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="13" t="s">
+      <c r="J3" s="15" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="16" t="s">
+      <c r="L3" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="13" t="s">
+      <c r="M3" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="N3" s="13" t="s">
+      <c r="N3" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="O3" s="13" t="s">
+      <c r="O3" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="P3" s="13" t="s">
+      <c r="P3" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="Q3" s="17" t="s">
+      <c r="Q3" s="19" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:17">
-      <c r="A4" s="18" t="s">
+      <c r="A4" s="20" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="18"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="21" t="s">
+      <c r="B4" s="20"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="23" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="22"/>
-      <c r="I4" s="21" t="s">
+      <c r="H4" s="24"/>
+      <c r="I4" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="23"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="24"/>
-      <c r="M4" s="25" t="s">
+      <c r="J4" s="25"/>
+      <c r="K4" s="24"/>
+      <c r="L4" s="26"/>
+      <c r="M4" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="25"/>
-      <c r="O4" s="25"/>
-      <c r="P4" s="25"/>
-      <c r="Q4" s="26"/>
+      <c r="N4" s="27"/>
+      <c r="O4" s="27"/>
+      <c r="P4" s="27"/>
+      <c r="Q4" s="28"/>
     </row>
     <row r="5" spans="1:17">
-      <c r="A5" s="27"/>
-      <c r="B5" s="27" t="s">
+      <c r="A5" s="29"/>
+      <c r="B5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="27" t="s">
+      <c r="C5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D5" s="27" t="s">
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="E5" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="28"/>
-      <c r="G5" s="29"/>
-      <c r="H5" s="30"/>
-      <c r="I5" s="29"/>
-      <c r="J5" s="31" t="b">
+      <c r="F5" s="30"/>
+      <c r="G5" s="31"/>
+      <c r="H5" s="32"/>
+      <c r="I5" s="31"/>
+      <c r="J5" s="33" t="b">
         <v>1</v>
       </c>
-      <c r="K5" s="30">
+      <c r="K5" s="32">
         <v>0.1</v>
       </c>
-      <c r="L5" s="29"/>
-      <c r="M5" s="31"/>
-      <c r="N5" s="31"/>
-      <c r="O5" s="31"/>
-      <c r="P5" s="31"/>
-      <c r="Q5" s="30"/>
+      <c r="L5" s="31"/>
+      <c r="M5" s="33"/>
+      <c r="N5" s="33"/>
+      <c r="O5" s="33"/>
+      <c r="P5" s="33"/>
+      <c r="Q5" s="32"/>
     </row>
     <row r="6" spans="1:17">
-      <c r="A6" s="27"/>
-      <c r="B6" s="27"/>
-      <c r="C6" s="27" t="s">
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="29" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="30"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="31"/>
+      <c r="J6" s="33" t="b">
+        <v>1</v>
+      </c>
+      <c r="K6" s="32">
+        <v>0.1</v>
+      </c>
+      <c r="L6" s="31"/>
+      <c r="M6" s="33"/>
+      <c r="N6" s="33"/>
+      <c r="O6" s="33"/>
+      <c r="P6" s="33"/>
+      <c r="Q6" s="32"/>
+    </row>
+    <row r="7" spans="1:17">
+      <c r="B7" s="34" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="E6" s="27" t="s">
-        <v>31</v>
-      </c>
-      <c r="F6" s="28"/>
-      <c r="G6" s="29"/>
-      <c r="H6" s="30"/>
-      <c r="I6" s="29"/>
-      <c r="J6" s="31" t="b">
+      <c r="F7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G7" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17">
+      <c r="C8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="K6" s="30">
-        <v>0.1</v>
-      </c>
-      <c r="L6" s="29"/>
-      <c r="M6" s="31"/>
-      <c r="N6" s="31"/>
-      <c r="O6" s="31"/>
-      <c r="P6" s="31"/>
-      <c r="Q6" s="30"/>
+      <c r="E8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="3">
+        <v>200</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>

<commit_message>
feat: Implement projectile system and enhance bow mechanics for improved combat dynamics
Introduced a new projectile system, including the Projectile class and factory for spawning projectiles with various configurations. Enhanced bow mechanics by adding the BowFireAbility and integrating projectile configurations into the bow's abilities. Updated XML and JSON files to reflect new projectile and bow configurations, ensuring better gameplay dynamics and modularity within the combat system. Additionally, added new timing abilities for enhanced gameplay interactions.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
   <si>
     <t>##var</t>
   </si>
@@ -85,6 +85,12 @@
     <t>aim_angle</t>
   </si>
   <si>
+    <t>projectile_config_id</t>
+  </si>
+  <si>
+    <t>projectile_level</t>
+  </si>
+  <si>
     <t>##type</t>
   </si>
   <si>
@@ -106,6 +112,9 @@
     <t>float</t>
   </si>
   <si>
+    <t>string?</t>
+  </si>
+  <si>
     <t>##</t>
   </si>
   <si>
@@ -131,6 +140,15 @@
   </si>
   <si>
     <t>armor_absorb_damage,0</t>
+  </si>
+  <si>
+    <t>bow</t>
+  </si>
+  <si>
+    <t>弓</t>
+  </si>
+  <si>
+    <t>arrow</t>
   </si>
 </sst>
 </file>
@@ -837,7 +855,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -851,6 +869,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
@@ -868,6 +889,9 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -878,6 +902,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -898,6 +925,9 @@
     <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -922,6 +952,9 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -938,6 +971,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1254,8 +1290,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:Q8"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14" outlineLevelRow="7"/>
+  <dimension ref="A1:S10"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="1"/>
     <col min="2" max="2" width="11.5454545454545" style="1" customWidth="1"/>
@@ -1271,261 +1307,368 @@
     <col min="14" max="14" width="14" style="1" customWidth="1"/>
     <col min="15" max="15" width="17.7272727272727" style="1" customWidth="1"/>
     <col min="16" max="16" width="20.1818181818182" style="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5454545454545" style="4" customWidth="1"/>
+    <col min="17" max="17" width="11.5454545454545" style="5" customWidth="1"/>
+    <col min="18" max="18" width="25.0909090909091" style="5" customWidth="1"/>
+    <col min="19" max="19" width="20.1818181818182" style="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:19">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="9"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="10"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="7"/>
+      <c r="K1" s="10"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="7"/>
+      <c r="N1" s="7"/>
+      <c r="O1" s="7"/>
+      <c r="P1" s="7"/>
+      <c r="Q1" s="11"/>
+      <c r="R1" s="11"/>
+      <c r="S1" s="10"/>
     </row>
-    <row r="2" spans="1:17">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:19">
+      <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="6"/>
+      <c r="C2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="J2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="K2" s="15" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="L2" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="M2" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="N2" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="O2" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="P2" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="Q2" s="15" t="s">
         <v>17</v>
       </c>
+      <c r="R2" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="S2" s="15" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="3" spans="1:17">
-      <c r="A3" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E3" s="16" t="s">
+    <row r="3" spans="1:19">
+      <c r="A3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="17" t="s">
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
+      <c r="D3" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="18" t="s">
-        <v>19</v>
-      </c>
-      <c r="H3" s="19" t="s">
-        <v>19</v>
-      </c>
-      <c r="I3" s="18" t="s">
+      <c r="E3" s="19" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="15" t="s">
+      <c r="F3" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="K3" s="19" t="s">
+      <c r="G3" s="21" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" s="22" t="s">
+        <v>21</v>
+      </c>
+      <c r="I3" s="21" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="18" t="s">
+      <c r="J3" s="18" t="s">
+        <v>25</v>
+      </c>
+      <c r="K3" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="L3" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="M3" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="N3" s="18" t="s">
+        <v>21</v>
+      </c>
+      <c r="O3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="P3" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q3" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="R3" s="23" t="s">
+        <v>27</v>
+      </c>
+      <c r="S3" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="M3" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="N3" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="O3" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="P3" s="15" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q3" s="19" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="4" spans="1:17">
-      <c r="A4" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="23" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" s="24"/>
-      <c r="I4" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="J4" s="25"/>
-      <c r="K4" s="24"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="27" t="s">
+    <row r="4" spans="1:19">
+      <c r="A4" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="N4" s="27"/>
-      <c r="O4" s="27"/>
-      <c r="P4" s="27"/>
-      <c r="Q4" s="28"/>
+      <c r="B4" s="24"/>
+      <c r="C4" s="24"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="26"/>
+      <c r="G4" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="28"/>
+      <c r="I4" s="27" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="29"/>
+      <c r="K4" s="28"/>
+      <c r="L4" s="30"/>
+      <c r="M4" s="31" t="s">
+        <v>31</v>
+      </c>
+      <c r="N4" s="31"/>
+      <c r="O4" s="31"/>
+      <c r="P4" s="31"/>
+      <c r="Q4" s="32"/>
+      <c r="R4" s="32"/>
+      <c r="S4" s="33"/>
     </row>
-    <row r="5" spans="1:17">
-      <c r="A5" s="29"/>
-      <c r="B5" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="29" t="s">
-        <v>29</v>
+    <row r="5" spans="1:19">
+      <c r="A5" s="34"/>
+      <c r="B5" s="34" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
-      <c r="E5" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="30"/>
-      <c r="G5" s="31"/>
-      <c r="H5" s="32"/>
-      <c r="I5" s="31"/>
-      <c r="J5" s="33" t="b">
+      <c r="E5" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="35"/>
+      <c r="G5" s="36"/>
+      <c r="H5" s="37"/>
+      <c r="I5" s="36"/>
+      <c r="J5" s="38" t="b">
         <v>1</v>
       </c>
-      <c r="K5" s="32">
+      <c r="K5" s="37">
         <v>0.1</v>
       </c>
-      <c r="L5" s="31"/>
-      <c r="M5" s="33"/>
-      <c r="N5" s="33"/>
-      <c r="O5" s="33"/>
-      <c r="P5" s="33"/>
-      <c r="Q5" s="32"/>
+      <c r="L5" s="36"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+      <c r="O5" s="38"/>
+      <c r="P5" s="38"/>
+      <c r="Q5" s="39"/>
+      <c r="R5" s="39"/>
+      <c r="S5" s="37"/>
     </row>
-    <row r="6" spans="1:17">
-      <c r="A6" s="29"/>
-      <c r="B6" s="29"/>
-      <c r="C6" s="29" t="s">
-        <v>29</v>
+    <row r="6" spans="1:19">
+      <c r="A6" s="34"/>
+      <c r="B6" s="34"/>
+      <c r="C6" s="34" t="s">
+        <v>32</v>
       </c>
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="E6" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="30"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="31"/>
-      <c r="J6" s="33" t="b">
+      <c r="E6" s="34" t="s">
+        <v>33</v>
+      </c>
+      <c r="F6" s="35"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="37"/>
+      <c r="I6" s="36"/>
+      <c r="J6" s="38" t="b">
         <v>1</v>
       </c>
-      <c r="K6" s="32">
+      <c r="K6" s="37">
         <v>0.1</v>
       </c>
-      <c r="L6" s="31"/>
-      <c r="M6" s="33"/>
-      <c r="N6" s="33"/>
-      <c r="O6" s="33"/>
-      <c r="P6" s="33"/>
-      <c r="Q6" s="32"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="38"/>
+      <c r="N6" s="38"/>
+      <c r="O6" s="38"/>
+      <c r="P6" s="38"/>
+      <c r="Q6" s="39"/>
+      <c r="R6" s="39"/>
+      <c r="S6" s="37"/>
     </row>
-    <row r="7" spans="1:17">
-      <c r="B7" s="34" t="s">
-        <v>31</v>
+    <row r="7" spans="1:19">
+      <c r="B7" s="40" t="s">
+        <v>34</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G7" s="3">
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:17">
+    <row r="8" spans="1:19">
       <c r="C8" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D8" s="1">
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="G8" s="3">
         <v>200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19">
+      <c r="B9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="1">
+        <v>0</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J9" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K9" s="4">
+        <v>2</v>
+      </c>
+      <c r="L9" s="3">
+        <v>360</v>
+      </c>
+      <c r="M9" s="1">
+        <v>1</v>
+      </c>
+      <c r="N9" s="1">
+        <v>3</v>
+      </c>
+      <c r="O9" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="P9" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="5">
+        <v>10</v>
+      </c>
+      <c r="R9" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S9" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19">
+      <c r="C10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="J10" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K10" s="4">
+        <v>2</v>
+      </c>
+      <c r="L10" s="3">
+        <v>360</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1</v>
+      </c>
+      <c r="N10" s="1">
+        <v>3</v>
+      </c>
+      <c r="O10" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="P10" s="1">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="5">
+        <v>10</v>
+      </c>
+      <c r="R10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="S10" s="4">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="C1:Q1"/>
+    <mergeCell ref="C1:S1"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="I4:K4"/>
   </mergeCells>

</xml_diff>

<commit_message>
feat: Update projectile and bow configurations for enhanced combat dynamics
Modified the projectile system by adding new configurations and enhancing the bow mechanics. Updated XML and JSON files to reflect changes in projectile properties, including damage and tracking abilities. Adjusted bow cooldown and shooting parameters for improved gameplay balance. Refactored related classes to support new configurations, ensuring better integration within the combat system.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="39">
   <si>
     <t>##var</t>
   </si>
@@ -110,9 +110,6 @@
   </si>
   <si>
     <t>float</t>
-  </si>
-  <si>
-    <t>string?</t>
   </si>
   <si>
     <t>##</t>
@@ -855,7 +852,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -869,9 +866,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
@@ -889,9 +883,6 @@
     <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -974,9 +965,6 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1307,258 +1295,258 @@
     <col min="14" max="14" width="14" style="1" customWidth="1"/>
     <col min="15" max="15" width="17.7272727272727" style="1" customWidth="1"/>
     <col min="16" max="16" width="20.1818181818182" style="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5454545454545" style="5" customWidth="1"/>
-    <col min="18" max="18" width="25.0909090909091" style="5" customWidth="1"/>
+    <col min="17" max="17" width="11.5454545454545" style="2" customWidth="1"/>
+    <col min="18" max="18" width="25.0909090909091" style="2" customWidth="1"/>
     <col min="19" max="19" width="20.1818181818182" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="10"/>
-      <c r="I1" s="9"/>
-      <c r="J1" s="7"/>
-      <c r="K1" s="10"/>
-      <c r="L1" s="9"/>
-      <c r="M1" s="7"/>
-      <c r="N1" s="7"/>
-      <c r="O1" s="7"/>
-      <c r="P1" s="7"/>
-      <c r="Q1" s="11"/>
-      <c r="R1" s="11"/>
-      <c r="S1" s="10"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="7"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="6"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="8"/>
+      <c r="M1" s="6"/>
+      <c r="N1" s="6"/>
+      <c r="O1" s="6"/>
+      <c r="P1" s="6"/>
+      <c r="Q1" s="7"/>
+      <c r="R1" s="7"/>
+      <c r="S1" s="9"/>
     </row>
     <row r="2" spans="1:19">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6" t="s">
+      <c r="B2" s="5"/>
+      <c r="C2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="F2" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="14" t="s">
+      <c r="G2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="15" t="s">
+      <c r="H2" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="14" t="s">
+      <c r="I2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="12" t="s">
+      <c r="J2" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="15" t="s">
+      <c r="K2" s="13" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="14" t="s">
+      <c r="L2" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="12" t="s">
+      <c r="M2" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="12" t="s">
+      <c r="N2" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="12" t="s">
+      <c r="P2" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="15" t="s">
+      <c r="Q2" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="16" t="s">
+      <c r="R2" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="15" t="s">
+      <c r="S2" s="13" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="3" spans="1:19">
-      <c r="A3" s="17" t="s">
+      <c r="A3" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="17"/>
-      <c r="C3" s="17"/>
-      <c r="D3" s="18" t="s">
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="E3" s="19" t="s">
+      <c r="E3" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="22" t="s">
+      <c r="H3" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="I3" s="21" t="s">
+      <c r="I3" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="J3" s="18" t="s">
+      <c r="J3" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="K3" s="22" t="s">
+      <c r="K3" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="L3" s="21" t="s">
+      <c r="L3" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="M3" s="18" t="s">
+      <c r="M3" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="N3" s="18" t="s">
+      <c r="N3" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="O3" s="18" t="s">
+      <c r="O3" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="P3" s="18" t="s">
+      <c r="P3" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="Q3" s="22" t="s">
+      <c r="Q3" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="R3" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="S3" s="22" t="s">
-        <v>24</v>
+      <c r="R3" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="S3" s="20" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:19">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="22" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="27" t="s">
+      <c r="H4" s="26"/>
+      <c r="I4" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="H4" s="28"/>
-      <c r="I4" s="27" t="s">
+      <c r="J4" s="27"/>
+      <c r="K4" s="26"/>
+      <c r="L4" s="28"/>
+      <c r="M4" s="29" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="29"/>
-      <c r="K4" s="28"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="31" t="s">
-        <v>31</v>
-      </c>
-      <c r="N4" s="31"/>
-      <c r="O4" s="31"/>
-      <c r="P4" s="31"/>
-      <c r="Q4" s="32"/>
-      <c r="R4" s="32"/>
-      <c r="S4" s="33"/>
+      <c r="N4" s="29"/>
+      <c r="O4" s="29"/>
+      <c r="P4" s="29"/>
+      <c r="Q4" s="30"/>
+      <c r="R4" s="30"/>
+      <c r="S4" s="31"/>
     </row>
     <row r="5" spans="1:19">
-      <c r="A5" s="34"/>
-      <c r="B5" s="34" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="34" t="s">
-        <v>32</v>
+      <c r="A5" s="32"/>
+      <c r="B5" s="32" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="32" t="s">
+        <v>31</v>
       </c>
       <c r="D5" s="1">
         <v>0</v>
       </c>
-      <c r="E5" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="F5" s="35"/>
-      <c r="G5" s="36"/>
-      <c r="H5" s="37"/>
-      <c r="I5" s="36"/>
-      <c r="J5" s="38" t="b">
+      <c r="E5" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="33"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
+      <c r="I5" s="34"/>
+      <c r="J5" s="36" t="b">
         <v>1</v>
       </c>
-      <c r="K5" s="37">
+      <c r="K5" s="35">
         <v>0.1</v>
       </c>
-      <c r="L5" s="36"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="38"/>
-      <c r="O5" s="38"/>
-      <c r="P5" s="38"/>
-      <c r="Q5" s="39"/>
-      <c r="R5" s="39"/>
-      <c r="S5" s="37"/>
+      <c r="L5" s="34"/>
+      <c r="M5" s="36"/>
+      <c r="N5" s="36"/>
+      <c r="O5" s="36"/>
+      <c r="P5" s="36"/>
+      <c r="Q5" s="37"/>
+      <c r="R5" s="37"/>
+      <c r="S5" s="35"/>
     </row>
     <row r="6" spans="1:19">
-      <c r="A6" s="34"/>
-      <c r="B6" s="34"/>
-      <c r="C6" s="34" t="s">
-        <v>32</v>
+      <c r="A6" s="32"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32" t="s">
+        <v>31</v>
       </c>
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="E6" s="34" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" s="35"/>
-      <c r="G6" s="36"/>
-      <c r="H6" s="37"/>
-      <c r="I6" s="36"/>
-      <c r="J6" s="38" t="b">
+      <c r="E6" s="32" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="33"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="34"/>
+      <c r="J6" s="36" t="b">
         <v>1</v>
       </c>
-      <c r="K6" s="37">
+      <c r="K6" s="35">
         <v>0.1</v>
       </c>
-      <c r="L6" s="36"/>
-      <c r="M6" s="38"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="38"/>
-      <c r="P6" s="38"/>
-      <c r="Q6" s="39"/>
-      <c r="R6" s="39"/>
-      <c r="S6" s="37"/>
+      <c r="L6" s="34"/>
+      <c r="M6" s="36"/>
+      <c r="N6" s="36"/>
+      <c r="O6" s="36"/>
+      <c r="P6" s="36"/>
+      <c r="Q6" s="37"/>
+      <c r="R6" s="37"/>
+      <c r="S6" s="35"/>
     </row>
     <row r="7" spans="1:19">
-      <c r="B7" s="40" t="s">
-        <v>34</v>
+      <c r="B7" s="1" t="s">
+        <v>33</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D7" s="1">
         <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="G7" s="3">
         <v>100</v>
@@ -1566,16 +1554,16 @@
     </row>
     <row r="8" spans="1:19">
       <c r="C8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D8" s="1">
         <v>1</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>36</v>
       </c>
       <c r="G8" s="3">
         <v>200</v>
@@ -1583,43 +1571,43 @@
     </row>
     <row r="9" spans="1:19">
       <c r="B9" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D9" s="1">
         <v>0</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J9" s="1" t="b">
         <v>1</v>
       </c>
       <c r="K9" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L9" s="3">
         <v>360</v>
       </c>
       <c r="M9" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N9" s="1">
         <v>3</v>
       </c>
       <c r="O9" s="1">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="P9" s="1">
         <v>5</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="2">
         <v>10</v>
       </c>
-      <c r="R9" s="5" t="s">
-        <v>39</v>
+      <c r="R9" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="S9" s="4">
         <v>0</v>
@@ -1627,40 +1615,40 @@
     </row>
     <row r="10" spans="1:19">
       <c r="C10" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D10" s="1">
         <v>1</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J10" s="1" t="b">
         <v>1</v>
       </c>
       <c r="K10" s="4">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L10" s="3">
         <v>360</v>
       </c>
       <c r="M10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N10" s="1">
         <v>3</v>
       </c>
       <c r="O10" s="1">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="P10" s="1">
         <v>5</v>
       </c>
-      <c r="Q10" s="5">
+      <c r="Q10" s="2">
         <v>10</v>
       </c>
-      <c r="R10" s="5" t="s">
-        <v>39</v>
+      <c r="R10" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="S10" s="4">
         <v>0</v>

</xml_diff>

<commit_message>
feat: Add new bow abilities and refactor weapon configurations
- Introduced BowAimAbilityConfig and BowFireAbilityConfig with necessary properties and deserialization logic.
- Updated BowLevelConfig to include references to BowAim and BowFire configurations.
- Refactored WeaponLevelConfig to utilize WeaponCalculateDamageAbilityConfig and WeaponCooldownAbilityConfig.
- Enhanced existing classes with new properties for damage calculations and cooldowns.
- Updated serialization checks to ensure proper data types for new configurations.
- Adjusted layout settings in Unity project for better UI management.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="65">
   <si>
     <t>##var</t>
   </si>
@@ -52,6 +52,27 @@
     <t>lst_ability</t>
   </si>
   <si>
+    <t>armor</t>
+  </si>
+  <si>
+    <t>calculate_damage</t>
+  </si>
+  <si>
+    <t>cooldown</t>
+  </si>
+  <si>
+    <t>sword_collision_attack</t>
+  </si>
+  <si>
+    <t>bow_aim</t>
+  </si>
+  <si>
+    <t>bow_fire</t>
+  </si>
+  <si>
+    <t>priority</t>
+  </si>
+  <si>
     <t>hp</t>
   </si>
   <si>
@@ -64,27 +85,27 @@
     <t>is_damage_by_velocity</t>
   </si>
   <si>
-    <t>cooldown</t>
+    <t>velocity_damage_factor</t>
   </si>
   <si>
     <t>rotate_speed</t>
   </si>
   <si>
+    <t>aim_angle</t>
+  </si>
+  <si>
+    <t>arrow_count</t>
+  </si>
+  <si>
+    <t>arrow_interval</t>
+  </si>
+  <si>
+    <t>arrow_angle_step</t>
+  </si>
+  <si>
     <t>shoot_type</t>
   </si>
   <si>
-    <t>arrow_count</t>
-  </si>
-  <si>
-    <t>arrow_interval</t>
-  </si>
-  <si>
-    <t>arrow_angle_step</t>
-  </si>
-  <si>
-    <t>aim_angle</t>
-  </si>
-  <si>
     <t>projectile_config_id</t>
   </si>
   <si>
@@ -106,22 +127,82 @@
     <t>int?</t>
   </si>
   <si>
+    <t>float</t>
+  </si>
+  <si>
     <t>bool</t>
   </si>
   <si>
-    <t>float</t>
-  </si>
-  <si>
     <t>##</t>
   </si>
   <si>
-    <t>armor</t>
-  </si>
-  <si>
-    <t>weapon</t>
-  </si>
-  <si>
-    <t>0:连射，1：散射</t>
+    <t>武器通用</t>
+  </si>
+  <si>
+    <t>近战武器</t>
+  </si>
+  <si>
+    <t>远程武器</t>
+  </si>
+  <si>
+    <t>防具血量</t>
+  </si>
+  <si>
+    <t>防具防御</t>
+  </si>
+  <si>
+    <t>攻击力</t>
+  </si>
+  <si>
+    <t>优先级</t>
+  </si>
+  <si>
+    <t>冷却时间</t>
+  </si>
+  <si>
+    <t>是否根据速度计算伤害</t>
+  </si>
+  <si>
+    <t>速度伤害倍率</t>
+  </si>
+  <si>
+    <t>瞄准速度</t>
+  </si>
+  <si>
+    <t>瞄准角度差</t>
+  </si>
+  <si>
+    <t>发射物数量</t>
+  </si>
+  <si>
+    <t>连射发射物时间间隔</t>
+  </si>
+  <si>
+    <t>散射发射物角度差</t>
+  </si>
+  <si>
+    <t>发射类型</t>
+  </si>
+  <si>
+    <t>发射物id</t>
+  </si>
+  <si>
+    <t>发射物等级</t>
+  </si>
+  <si>
+    <t>不填则表示使用球的攻击力</t>
+  </si>
+  <si>
+    <t>远程：射击间隔
+近战：伤害间隔
+防止武器一秒砍人20刀</t>
+  </si>
+  <si>
+    <t>最终伤害=伤害x相对速度x倍率</t>
+  </si>
+  <si>
+    <t>0:连射
+1：散射</t>
   </si>
   <si>
     <t>sword</t>
@@ -136,7 +217,7 @@
     <t>盾</t>
   </si>
   <si>
-    <t>armor_absorb_damage,0</t>
+    <t>armor_absorb_damage</t>
   </si>
   <si>
     <t>bow</t>
@@ -538,7 +619,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -578,6 +659,30 @@
       <left style="medium">
         <color auto="1"/>
       </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -593,6 +698,32 @@
       <left style="thin">
         <color auto="1"/>
       </left>
+      <right style="medium">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
       <right style="medium">
         <color auto="1"/>
       </right>
@@ -728,7 +859,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="5">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
@@ -740,34 +871,34 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="10">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="13">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="14">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="15">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="16">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
@@ -852,10 +983,13 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -868,34 +1002,70 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -919,6 +1089,15 @@
     <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -931,13 +1110,40 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
@@ -946,8 +1152,50 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
@@ -958,10 +1206,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1">
@@ -1278,387 +1538,686 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S10"/>
+  <dimension ref="A1:AA13"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="9" style="1"/>
-    <col min="2" max="2" width="11.5454545454545" style="1" customWidth="1"/>
-    <col min="3" max="5" width="9" style="1"/>
-    <col min="6" max="6" width="33.6363636363636" style="2" customWidth="1"/>
-    <col min="7" max="7" width="9" style="3"/>
-    <col min="8" max="8" width="9" style="4"/>
-    <col min="9" max="9" width="8.09090909090909" style="3" customWidth="1"/>
-    <col min="10" max="10" width="26.2727272727273" style="1" customWidth="1"/>
-    <col min="11" max="11" width="10.3636363636364" style="4" customWidth="1"/>
-    <col min="12" max="12" width="15.2727272727273" style="3" customWidth="1"/>
-    <col min="13" max="13" width="18.3636363636364" style="1" customWidth="1"/>
-    <col min="14" max="14" width="14" style="1" customWidth="1"/>
-    <col min="15" max="15" width="17.7272727272727" style="1" customWidth="1"/>
-    <col min="16" max="16" width="20.1818181818182" style="1" customWidth="1"/>
-    <col min="17" max="17" width="11.5454545454545" style="2" customWidth="1"/>
-    <col min="18" max="18" width="25.0909090909091" style="2" customWidth="1"/>
-    <col min="19" max="19" width="20.1818181818182" style="4" customWidth="1"/>
+    <col min="1" max="1" width="9" style="2"/>
+    <col min="2" max="2" width="11.5454545454545" style="2" customWidth="1"/>
+    <col min="3" max="5" width="9" style="2"/>
+    <col min="6" max="6" width="33.6363636363636" style="3" customWidth="1"/>
+    <col min="7" max="7" width="23.8181818181818" style="4" customWidth="1"/>
+    <col min="8" max="8" width="10.3636363636364" style="2" hidden="1" customWidth="1"/>
+    <col min="9" max="9" width="9.90909090909091" style="5" customWidth="1"/>
+    <col min="10" max="10" width="9.90909090909091" style="3" customWidth="1"/>
+    <col min="11" max="11" width="20.1818181818182" style="6" customWidth="1"/>
+    <col min="12" max="12" width="10.3636363636364" style="5" hidden="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1818181818182" style="2" customWidth="1"/>
+    <col min="14" max="14" width="10.3636363636364" style="5" customWidth="1"/>
+    <col min="15" max="15" width="26.2727272727273" style="6" customWidth="1"/>
+    <col min="16" max="16" width="27.5454545454545" style="2" customWidth="1"/>
+    <col min="17" max="17" width="10.3636363636364" style="7" hidden="1" customWidth="1"/>
+    <col min="18" max="18" width="15.2727272727273" style="8" customWidth="1"/>
+    <col min="19" max="19" width="18.3636363636364" style="2" customWidth="1"/>
+    <col min="20" max="20" width="14" style="2" hidden="1" customWidth="1"/>
+    <col min="21" max="21" width="14" style="2" customWidth="1"/>
+    <col min="22" max="22" width="21.7272727272727" style="2" customWidth="1"/>
+    <col min="23" max="23" width="20.1818181818182" style="2" customWidth="1"/>
+    <col min="24" max="24" width="11.5454545454545" style="3" customWidth="1"/>
+    <col min="25" max="25" width="25.0909090909091" style="3" customWidth="1"/>
+    <col min="26" max="26" width="25.0909090909091" style="9" customWidth="1"/>
+    <col min="27" max="27" width="20.1818181818182" style="7" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19">
-      <c r="A1" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="5" t="s">
+    <row r="1" spans="1:27">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="11" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="8"/>
-      <c r="H1" s="9"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="6"/>
-      <c r="K1" s="9"/>
-      <c r="L1" s="8"/>
-      <c r="M1" s="6"/>
-      <c r="N1" s="6"/>
-      <c r="O1" s="6"/>
-      <c r="P1" s="6"/>
-      <c r="Q1" s="7"/>
-      <c r="R1" s="7"/>
-      <c r="S1" s="9"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="12"/>
+      <c r="M1" s="13"/>
+      <c r="N1" s="12"/>
+      <c r="O1" s="14"/>
+      <c r="P1" s="13"/>
+      <c r="Q1" s="15"/>
+      <c r="R1" s="12"/>
+      <c r="S1" s="12"/>
+      <c r="T1" s="12"/>
+      <c r="U1" s="12"/>
+      <c r="V1" s="12"/>
+      <c r="W1" s="12"/>
+      <c r="X1" s="12"/>
+      <c r="Y1" s="12"/>
+      <c r="Z1" s="12"/>
+      <c r="AA1" s="16"/>
     </row>
-    <row r="2" spans="1:19">
-      <c r="A2" s="5" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5" t="s">
+    <row r="2" spans="1:27">
+      <c r="A2" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="10" t="s">
+      <c r="D2" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="11" t="s">
+      <c r="F2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="12" t="s">
+      <c r="G2" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="H2" s="20"/>
+      <c r="I2" s="21"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="L2" s="12"/>
+      <c r="M2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="J2" s="10" t="s">
+      <c r="N2" s="12"/>
+      <c r="O2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="K2" s="13" t="s">
+      <c r="P2" s="13"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="L2" s="12" t="s">
+      <c r="S2" s="12"/>
+      <c r="T2" s="12"/>
+      <c r="U2" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="M2" s="10" t="s">
+      <c r="V2" s="12"/>
+      <c r="W2" s="12"/>
+      <c r="X2" s="12"/>
+      <c r="Y2" s="12"/>
+      <c r="Z2" s="12"/>
+      <c r="AA2" s="16"/>
+    </row>
+    <row r="3" spans="1:27">
+      <c r="A3" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="N2" s="10" t="s">
+      <c r="I3" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="O2" s="10" t="s">
+      <c r="J3" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="P2" s="10" t="s">
+      <c r="K3" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" s="13" t="s">
+      <c r="L3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="N3" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="O3" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="R2" s="14" t="s">
+      <c r="P3" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="S2" s="13" t="s">
+      <c r="Q3" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="R3" s="26" t="s">
         <v>19</v>
       </c>
+      <c r="S3" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="T3" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="U3" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="V3" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="W3" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="X3" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y3" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="Z3" s="27" t="s">
+        <v>26</v>
+      </c>
+      <c r="AA3" s="15" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="3" spans="1:19">
-      <c r="A3" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="D3" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="17" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="18" t="s">
-        <v>23</v>
-      </c>
-      <c r="G3" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="I3" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="J3" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="K3" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="L3" s="19" t="s">
-        <v>26</v>
-      </c>
-      <c r="M3" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="N3" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="O3" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="P3" s="16" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q3" s="20" t="s">
-        <v>26</v>
-      </c>
-      <c r="R3" s="21" t="s">
-        <v>22</v>
-      </c>
-      <c r="S3" s="20" t="s">
-        <v>21</v>
+    <row r="4" spans="1:27">
+      <c r="A4" s="28" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="32"/>
+      <c r="H4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="K4" s="35" t="s">
+        <v>31</v>
+      </c>
+      <c r="L4" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="M4" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="N4" s="33" t="s">
+        <v>28</v>
+      </c>
+      <c r="O4" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="P4" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="Q4" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="R4" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="S4" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="U4" s="29" t="s">
+        <v>28</v>
+      </c>
+      <c r="V4" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="W4" s="29" t="s">
+        <v>32</v>
+      </c>
+      <c r="X4" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="Y4" s="34" t="s">
+        <v>29</v>
+      </c>
+      <c r="Z4" s="36" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA4" s="36" t="s">
+        <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:19">
-      <c r="A4" s="22" t="s">
-        <v>27</v>
-      </c>
-      <c r="B4" s="22"/>
-      <c r="C4" s="22"/>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="24"/>
-      <c r="G4" s="25" t="s">
-        <v>28</v>
-      </c>
-      <c r="H4" s="26"/>
-      <c r="I4" s="25" t="s">
-        <v>29</v>
-      </c>
-      <c r="J4" s="27"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="28"/>
-      <c r="M4" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="N4" s="29"/>
-      <c r="O4" s="29"/>
-      <c r="P4" s="29"/>
-      <c r="Q4" s="30"/>
-      <c r="R4" s="30"/>
-      <c r="S4" s="31"/>
+    <row r="5" spans="1:27">
+      <c r="A5" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="39"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="41" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="42"/>
+      <c r="I5" s="43"/>
+      <c r="J5" s="44"/>
+      <c r="K5" s="45" t="s">
+        <v>35</v>
+      </c>
+      <c r="L5" s="46"/>
+      <c r="M5" s="47"/>
+      <c r="N5" s="46"/>
+      <c r="O5" s="45" t="s">
+        <v>36</v>
+      </c>
+      <c r="P5" s="46"/>
+      <c r="Q5" s="48"/>
+      <c r="R5" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="S5" s="49"/>
+      <c r="T5" s="49"/>
+      <c r="U5" s="49"/>
+      <c r="V5" s="49"/>
+      <c r="W5" s="49"/>
+      <c r="X5" s="49"/>
+      <c r="Y5" s="49"/>
+      <c r="Z5" s="49"/>
+      <c r="AA5" s="50"/>
     </row>
-    <row r="5" spans="1:19">
-      <c r="A5" s="32"/>
-      <c r="B5" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="C5" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="33"/>
-      <c r="G5" s="34"/>
-      <c r="H5" s="35"/>
-      <c r="I5" s="34"/>
-      <c r="J5" s="36" t="b">
+    <row r="6" spans="1:27">
+      <c r="A6" s="38" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="39"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="42"/>
+      <c r="I6" s="43" t="s">
+        <v>38</v>
+      </c>
+      <c r="J6" s="44" t="s">
+        <v>39</v>
+      </c>
+      <c r="K6" s="51" t="s">
+        <v>40</v>
+      </c>
+      <c r="L6" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="M6" s="42" t="s">
+        <v>42</v>
+      </c>
+      <c r="N6" s="43" t="s">
+        <v>41</v>
+      </c>
+      <c r="O6" s="51" t="s">
+        <v>43</v>
+      </c>
+      <c r="P6" s="42" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q6" s="52" t="s">
+        <v>41</v>
+      </c>
+      <c r="R6" s="53" t="s">
+        <v>45</v>
+      </c>
+      <c r="S6" s="54" t="s">
+        <v>46</v>
+      </c>
+      <c r="T6" s="52" t="s">
+        <v>41</v>
+      </c>
+      <c r="U6" s="54" t="s">
+        <v>47</v>
+      </c>
+      <c r="V6" s="54" t="s">
+        <v>48</v>
+      </c>
+      <c r="W6" s="54" t="s">
+        <v>49</v>
+      </c>
+      <c r="X6" s="55" t="s">
+        <v>50</v>
+      </c>
+      <c r="Y6" s="55" t="s">
+        <v>51</v>
+      </c>
+      <c r="Z6" s="56" t="s">
+        <v>52</v>
+      </c>
+      <c r="AA6" s="52" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="57" customHeight="1" spans="1:27">
+      <c r="A7" s="57" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="57"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="59"/>
+      <c r="G7" s="60"/>
+      <c r="H7" s="61" t="s">
+        <v>41</v>
+      </c>
+      <c r="I7" s="62"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="L7" s="62"/>
+      <c r="M7" s="61" t="s">
+        <v>54</v>
+      </c>
+      <c r="N7" s="62"/>
+      <c r="O7" s="64"/>
+      <c r="P7" s="61" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q7" s="65"/>
+      <c r="R7" s="66"/>
+      <c r="S7" s="67"/>
+      <c r="T7" s="67"/>
+      <c r="U7" s="67"/>
+      <c r="V7" s="67"/>
+      <c r="W7" s="67"/>
+      <c r="X7" s="68" t="s">
+        <v>56</v>
+      </c>
+      <c r="Y7" s="68"/>
+      <c r="Z7" s="69"/>
+      <c r="AA7" s="70"/>
+    </row>
+    <row r="8" spans="1:27">
+      <c r="A8" s="71"/>
+      <c r="B8" s="71" t="s">
+        <v>57</v>
+      </c>
+      <c r="C8" s="71" t="s">
+        <v>57</v>
+      </c>
+      <c r="D8" s="2">
+        <v>0</v>
+      </c>
+      <c r="E8" s="71" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="72"/>
+      <c r="G8" s="73"/>
+      <c r="H8" s="74"/>
+      <c r="I8" s="75"/>
+      <c r="J8" s="76"/>
+      <c r="K8" s="77"/>
+      <c r="L8" s="75">
+        <v>0</v>
+      </c>
+      <c r="M8" s="74">
+        <v>0.1</v>
+      </c>
+      <c r="N8" s="75">
+        <v>0</v>
+      </c>
+      <c r="O8" s="77" t="b">
         <v>1</v>
       </c>
-      <c r="K5" s="35">
+      <c r="P8" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="Q8" s="78">
+        <v>0</v>
+      </c>
+      <c r="R8" s="79"/>
+      <c r="S8" s="74"/>
+      <c r="T8" s="74"/>
+      <c r="U8" s="74"/>
+      <c r="V8" s="74"/>
+      <c r="W8" s="74"/>
+      <c r="X8" s="76"/>
+      <c r="Y8" s="76"/>
+      <c r="Z8" s="80"/>
+      <c r="AA8" s="78"/>
+    </row>
+    <row r="9" spans="1:27">
+      <c r="A9" s="71"/>
+      <c r="B9" s="71"/>
+      <c r="C9" s="71" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1</v>
+      </c>
+      <c r="E9" s="71" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="72"/>
+      <c r="G9" s="73"/>
+      <c r="H9" s="74"/>
+      <c r="I9" s="75"/>
+      <c r="J9" s="76"/>
+      <c r="K9" s="77"/>
+      <c r="L9" s="75">
+        <v>0</v>
+      </c>
+      <c r="M9" s="74">
         <v>0.1</v>
       </c>
-      <c r="L5" s="34"/>
-      <c r="M5" s="36"/>
-      <c r="N5" s="36"/>
-      <c r="O5" s="36"/>
-      <c r="P5" s="36"/>
-      <c r="Q5" s="37"/>
-      <c r="R5" s="37"/>
-      <c r="S5" s="35"/>
+      <c r="N9" s="75">
+        <v>0</v>
+      </c>
+      <c r="O9" s="77" t="b">
+        <v>1</v>
+      </c>
+      <c r="P9" s="2">
+        <v>0.05</v>
+      </c>
+      <c r="Q9" s="78">
+        <v>0</v>
+      </c>
+      <c r="R9" s="79"/>
+      <c r="S9" s="74"/>
+      <c r="T9" s="74"/>
+      <c r="U9" s="74"/>
+      <c r="V9" s="74"/>
+      <c r="W9" s="74"/>
+      <c r="X9" s="76"/>
+      <c r="Y9" s="76"/>
+      <c r="Z9" s="80"/>
+      <c r="AA9" s="78"/>
     </row>
-    <row r="6" spans="1:19">
-      <c r="A6" s="32"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32" t="s">
-        <v>31</v>
-      </c>
-      <c r="D6" s="1">
+    <row r="10" spans="1:27">
+      <c r="B10" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2">
+        <v>0</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
+      <c r="I10" s="5">
+        <v>100</v>
+      </c>
+      <c r="J10" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2">
         <v>1</v>
       </c>
-      <c r="E6" s="32" t="s">
-        <v>32</v>
-      </c>
-      <c r="F6" s="33"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="34"/>
-      <c r="J6" s="36" t="b">
+      <c r="E11" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="3"/>
+      <c r="G11" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="2">
+        <v>0</v>
+      </c>
+      <c r="I11" s="5">
+        <v>200</v>
+      </c>
+      <c r="J11" s="3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="B12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D12" s="2">
+        <v>0</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="L12" s="5">
+        <v>0</v>
+      </c>
+      <c r="M12" s="2">
+        <v>5</v>
+      </c>
+      <c r="N12" s="5">
+        <v>0</v>
+      </c>
+      <c r="O12" s="6"/>
+      <c r="R12" s="8">
+        <v>360</v>
+      </c>
+      <c r="S12" s="2">
+        <v>10</v>
+      </c>
+      <c r="T12" s="5">
+        <v>0</v>
+      </c>
+      <c r="U12" s="2">
+        <v>3</v>
+      </c>
+      <c r="V12" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="W12" s="2">
+        <v>5</v>
+      </c>
+      <c r="X12" s="3">
         <v>1</v>
       </c>
-      <c r="K6" s="35">
+      <c r="Y12" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z12" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA12" s="7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:27">
+      <c r="C13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="2">
+        <v>1</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="L13" s="5">
+        <v>0</v>
+      </c>
+      <c r="M13" s="2">
+        <v>5</v>
+      </c>
+      <c r="N13" s="5">
+        <v>0</v>
+      </c>
+      <c r="O13" s="6"/>
+      <c r="R13" s="8">
+        <v>360</v>
+      </c>
+      <c r="S13" s="2">
+        <v>10</v>
+      </c>
+      <c r="T13" s="5">
+        <v>0</v>
+      </c>
+      <c r="U13" s="2">
+        <v>3</v>
+      </c>
+      <c r="V13" s="2">
         <v>0.1</v>
       </c>
-      <c r="L6" s="34"/>
-      <c r="M6" s="36"/>
-      <c r="N6" s="36"/>
-      <c r="O6" s="36"/>
-      <c r="P6" s="36"/>
-      <c r="Q6" s="37"/>
-      <c r="R6" s="37"/>
-      <c r="S6" s="35"/>
-    </row>
-    <row r="7" spans="1:19">
-      <c r="B7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G7" s="3">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19">
-      <c r="C8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="1">
+      <c r="W13" s="2">
+        <v>5</v>
+      </c>
+      <c r="X13" s="3">
         <v>1</v>
       </c>
-      <c r="E8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" s="3">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="9" spans="1:19">
-      <c r="B9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K9" s="4">
-        <v>5</v>
-      </c>
-      <c r="L9" s="3">
-        <v>360</v>
-      </c>
-      <c r="M9" s="1">
-        <v>0</v>
-      </c>
-      <c r="N9" s="1">
-        <v>3</v>
-      </c>
-      <c r="O9" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="P9" s="1">
-        <v>5</v>
-      </c>
-      <c r="Q9" s="2">
-        <v>10</v>
-      </c>
-      <c r="R9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S9" s="4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:19">
-      <c r="C10" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" s="1">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J10" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K10" s="4">
-        <v>5</v>
-      </c>
-      <c r="L10" s="3">
-        <v>360</v>
-      </c>
-      <c r="M10" s="1">
-        <v>0</v>
-      </c>
-      <c r="N10" s="1">
-        <v>3</v>
-      </c>
-      <c r="O10" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="P10" s="1">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="2">
-        <v>10</v>
-      </c>
-      <c r="R10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S10" s="4">
+      <c r="Y13" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="Z13" s="7">
+        <v>0</v>
+      </c>
+      <c r="AA13" s="7">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="C1:S1"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:K4"/>
+  <mergeCells count="11">
+    <mergeCell ref="C1:AA1"/>
+    <mergeCell ref="G2:J2"/>
+    <mergeCell ref="K2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="O2:Q2"/>
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="U2:AA2"/>
+    <mergeCell ref="G5:J5"/>
+    <mergeCell ref="K5:N5"/>
+    <mergeCell ref="O5:Q5"/>
+    <mergeCell ref="R5:AA5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>

</xml_diff>

<commit_message>
feat: Update equipment prefabs and configuration files for improved combat mechanics
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -1986,7 +1986,7 @@
         <v>1</v>
       </c>
       <c r="P8" s="2">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="Q8" s="78">
         <v>0</v>
@@ -2033,7 +2033,7 @@
         <v>1</v>
       </c>
       <c r="P9" s="2">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="Q9" s="78">
         <v>0</v>

</xml_diff>

<commit_message>
feat: Introduce advanced elicitation and brainstorming skills with structured workflows
- Added new skills for advanced elicitation and brainstorming, enabling deeper critique and creative ideation.
- Included comprehensive methods in CSV format for collaboration, advanced reasoning, competitive analysis, and creative exploration.
- Developed structured workflows and templates to facilitate effective brainstorming sessions.
- Enhanced documentation in SKILL.md and workflow files to guide users through the new features and techniques.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -419,30 +419,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF92D050"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -889,7 +871,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="9">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="9">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0">
@@ -913,16 +895,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="9" borderId="12">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="13">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="12">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="11" borderId="14">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="13">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="12">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="14">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="15">
@@ -931,89 +913,89 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="16">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0">
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="10" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="15" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="16" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="19" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="23" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="24" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="27" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="28" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="31" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0">
+    <xf numFmtId="0" fontId="20" fillId="32" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="0">
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="35" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="36" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="37" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="38" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1044,193 +1026,151 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="1" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1239,52 +1179,31 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="2" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1670,7 +1589,7 @@
       <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="14"/>
+      <c r="B2" s="10"/>
       <c r="C2" s="10" t="s">
         <v>3</v>
       </c>
@@ -1680,46 +1599,46 @@
       <c r="E2" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="F2" s="15" t="s">
+      <c r="F2" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G2" s="16" t="s">
+      <c r="G2" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="H2" s="17" t="s">
+      <c r="H2" s="16" t="s">
         <v>8</v>
       </c>
-      <c r="I2" s="18"/>
-      <c r="J2" s="18"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="20" t="s">
+      <c r="I2" s="17"/>
+      <c r="J2" s="17"/>
+      <c r="K2" s="18"/>
+      <c r="L2" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="M2" s="21"/>
-      <c r="N2" s="20" t="s">
+      <c r="M2" s="20"/>
+      <c r="N2" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="O2" s="21"/>
-      <c r="P2" s="22" t="s">
+      <c r="O2" s="20"/>
+      <c r="P2" s="12" t="s">
         <v>11</v>
       </c>
       <c r="Q2" s="12"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="24" t="s">
+      <c r="R2" s="12"/>
+      <c r="S2" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="T2" s="25"/>
-      <c r="U2" s="26"/>
-      <c r="V2" s="24" t="s">
+      <c r="T2" s="22"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="W2" s="25"/>
-      <c r="X2" s="25"/>
-      <c r="Y2" s="25"/>
-      <c r="Z2" s="25"/>
-      <c r="AA2" s="25"/>
-      <c r="AB2" s="26"/>
-      <c r="AC2" s="27" t="s">
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
+      <c r="Y2" s="22"/>
+      <c r="Z2" s="22"/>
+      <c r="AA2" s="22"/>
+      <c r="AB2" s="23"/>
+      <c r="AC2" s="24" t="s">
         <v>14</v>
       </c>
     </row>
@@ -1727,17 +1646,17 @@
       <c r="A3" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="14"/>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="15" t="s">
+      <c r="B3" s="10"/>
+      <c r="C3" s="10"/>
+      <c r="D3" s="10"/>
+      <c r="E3" s="10"/>
+      <c r="F3" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="G3" s="16" t="s">
+      <c r="G3" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="28" t="s">
+      <c r="H3" s="25" t="s">
         <v>3</v>
       </c>
       <c r="I3" s="10" t="s">
@@ -1746,40 +1665,40 @@
       <c r="J3" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="K3" s="29" t="s">
+      <c r="K3" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="L3" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="M3" s="19" t="s">
+      <c r="M3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="N3" s="28" t="s">
+      <c r="N3" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="O3" s="19" t="s">
+      <c r="O3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="30" t="s">
+      <c r="P3" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="Q3" s="18" t="s">
+      <c r="Q3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="R3" s="31" t="s">
+      <c r="R3" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="S3" s="28" t="s">
+      <c r="S3" s="25" t="s">
         <v>21</v>
       </c>
       <c r="T3" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="U3" s="19" t="s">
+      <c r="U3" s="18" t="s">
         <v>15</v>
       </c>
-      <c r="V3" s="28" t="s">
+      <c r="V3" s="25" t="s">
         <v>23</v>
       </c>
       <c r="W3" s="10" t="s">
@@ -1797,260 +1716,260 @@
       <c r="AA3" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="AB3" s="29" t="s">
+      <c r="AB3" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="AC3" s="32"/>
+      <c r="AC3" s="24"/>
     </row>
     <row r="4" s="2" customFormat="1" spans="1:29">
-      <c r="A4" s="33" t="s">
+      <c r="A4" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="B4" s="34"/>
-      <c r="C4" s="34"/>
-      <c r="D4" s="35" t="s">
+      <c r="B4" s="27"/>
+      <c r="C4" s="27"/>
+      <c r="D4" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="36" t="s">
+      <c r="E4" s="29" t="s">
         <v>31</v>
       </c>
-      <c r="F4" s="37" t="s">
+      <c r="F4" s="30" t="s">
         <v>30</v>
       </c>
-      <c r="G4" s="38" t="s">
+      <c r="G4" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="39"/>
-      <c r="I4" s="35" t="s">
+      <c r="H4" s="32"/>
+      <c r="I4" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="J4" s="35" t="s">
+      <c r="J4" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="K4" s="40" t="s">
+      <c r="K4" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="L4" s="41" t="s">
+      <c r="L4" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="M4" s="40" t="s">
+      <c r="M4" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="N4" s="41" t="s">
+      <c r="N4" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="O4" s="40" t="s">
+      <c r="O4" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="P4" s="42" t="s">
+      <c r="P4" s="34" t="s">
         <v>34</v>
       </c>
-      <c r="Q4" s="35" t="s">
+      <c r="Q4" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="R4" s="43" t="s">
+      <c r="R4" s="35" t="s">
         <v>30</v>
       </c>
-      <c r="S4" s="41" t="s">
+      <c r="S4" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="T4" s="35" t="s">
+      <c r="T4" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="U4" s="40" t="s">
+      <c r="U4" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="V4" s="41" t="s">
+      <c r="V4" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="W4" s="35" t="s">
+      <c r="W4" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="X4" s="35" t="s">
+      <c r="X4" s="28" t="s">
         <v>33</v>
       </c>
-      <c r="Y4" s="35" t="s">
+      <c r="Y4" s="28" t="s">
         <v>35</v>
       </c>
-      <c r="Z4" s="35" t="s">
+      <c r="Z4" s="28" t="s">
         <v>31</v>
       </c>
-      <c r="AA4" s="35" t="s">
+      <c r="AA4" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="AB4" s="40" t="s">
+      <c r="AB4" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="AC4" s="44" t="s">
+      <c r="AC4" s="36" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="5" s="3" customFormat="1" spans="1:29">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="B5" s="46"/>
-      <c r="C5" s="46"/>
-      <c r="D5" s="47"/>
-      <c r="E5" s="48"/>
-      <c r="F5" s="49"/>
-      <c r="G5" s="50"/>
-      <c r="H5" s="51" t="s">
+      <c r="B5" s="37"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="39"/>
+      <c r="F5" s="40"/>
+      <c r="G5" s="41"/>
+      <c r="H5" s="42" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="52"/>
-      <c r="J5" s="52"/>
-      <c r="K5" s="53"/>
-      <c r="L5" s="54" t="s">
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="43"/>
+      <c r="L5" s="44" t="s">
         <v>38</v>
       </c>
-      <c r="M5" s="55"/>
-      <c r="N5" s="55"/>
-      <c r="O5" s="56"/>
-      <c r="P5" s="55" t="s">
+      <c r="M5" s="45"/>
+      <c r="N5" s="45"/>
+      <c r="O5" s="46"/>
+      <c r="P5" s="45" t="s">
         <v>39</v>
       </c>
-      <c r="Q5" s="55"/>
-      <c r="R5" s="57"/>
-      <c r="S5" s="54" t="s">
+      <c r="Q5" s="45"/>
+      <c r="R5" s="45"/>
+      <c r="S5" s="44" t="s">
         <v>40</v>
       </c>
-      <c r="T5" s="55"/>
-      <c r="U5" s="56"/>
-      <c r="V5" s="58"/>
-      <c r="W5" s="59"/>
-      <c r="X5" s="59"/>
-      <c r="Y5" s="59"/>
-      <c r="Z5" s="59"/>
-      <c r="AA5" s="59"/>
-      <c r="AB5" s="53"/>
-      <c r="AC5" s="60"/>
+      <c r="T5" s="45"/>
+      <c r="U5" s="46"/>
+      <c r="V5" s="47"/>
+      <c r="W5" s="48"/>
+      <c r="X5" s="48"/>
+      <c r="Y5" s="48"/>
+      <c r="Z5" s="48"/>
+      <c r="AA5" s="48"/>
+      <c r="AB5" s="43"/>
+      <c r="AC5" s="49"/>
     </row>
     <row r="6" s="3" customFormat="1" spans="1:29">
-      <c r="A6" s="45" t="s">
+      <c r="A6" s="37" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="46"/>
-      <c r="C6" s="46"/>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="49"/>
-      <c r="G6" s="50"/>
-      <c r="H6" s="61"/>
-      <c r="I6" s="62" t="s">
+      <c r="B6" s="37"/>
+      <c r="C6" s="37"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="40"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="50"/>
+      <c r="I6" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="J6" s="63" t="s">
+      <c r="J6" s="52" t="s">
         <v>42</v>
       </c>
-      <c r="K6" s="64" t="s">
+      <c r="K6" s="53" t="s">
         <v>43</v>
       </c>
-      <c r="L6" s="65" t="s">
+      <c r="L6" s="50" t="s">
         <v>44</v>
       </c>
-      <c r="M6" s="64" t="s">
+      <c r="M6" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="N6" s="65" t="s">
+      <c r="N6" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="O6" s="64" t="s">
+      <c r="O6" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="P6" s="66" t="s">
+      <c r="P6" s="54" t="s">
         <v>46</v>
       </c>
-      <c r="Q6" s="63" t="s">
+      <c r="Q6" s="52" t="s">
         <v>47</v>
       </c>
-      <c r="R6" s="67" t="s">
+      <c r="R6" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="S6" s="68" t="s">
+      <c r="S6" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="T6" s="69" t="s">
+      <c r="T6" s="40" t="s">
         <v>49</v>
       </c>
-      <c r="U6" s="64" t="s">
+      <c r="U6" s="53" t="s">
         <v>41</v>
       </c>
-      <c r="V6" s="68" t="s">
+      <c r="V6" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="W6" s="69" t="s">
+      <c r="W6" s="40" t="s">
         <v>51</v>
       </c>
-      <c r="X6" s="69" t="s">
+      <c r="X6" s="40" t="s">
         <v>52</v>
       </c>
-      <c r="Y6" s="69" t="s">
+      <c r="Y6" s="40" t="s">
         <v>53</v>
       </c>
-      <c r="Z6" s="69" t="s">
+      <c r="Z6" s="40" t="s">
         <v>54</v>
       </c>
-      <c r="AA6" s="69" t="s">
+      <c r="AA6" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="AB6" s="70" t="s">
+      <c r="AB6" s="57" t="s">
         <v>41</v>
       </c>
-      <c r="AC6" s="71"/>
+      <c r="AC6" s="58"/>
     </row>
     <row r="7" s="4" customFormat="1" ht="57" customHeight="1" spans="1:29">
-      <c r="A7" s="72" t="s">
+      <c r="A7" s="59" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="73"/>
-      <c r="C7" s="73"/>
-      <c r="D7" s="74"/>
-      <c r="E7" s="74"/>
-      <c r="F7" s="75"/>
-      <c r="G7" s="76"/>
-      <c r="H7" s="77"/>
-      <c r="J7" s="78"/>
-      <c r="K7" s="79"/>
-      <c r="L7" s="80" t="s">
+      <c r="B7" s="59"/>
+      <c r="C7" s="59"/>
+      <c r="D7" s="60"/>
+      <c r="E7" s="60"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="62"/>
+      <c r="H7" s="63"/>
+      <c r="J7" s="51"/>
+      <c r="K7" s="64"/>
+      <c r="L7" s="63" t="s">
         <v>56</v>
       </c>
-      <c r="M7" s="79"/>
-      <c r="N7" s="80" t="s">
+      <c r="M7" s="64"/>
+      <c r="N7" s="63" t="s">
         <v>57</v>
       </c>
-      <c r="O7" s="79"/>
-      <c r="P7" s="81"/>
-      <c r="Q7" s="62" t="s">
+      <c r="O7" s="64"/>
+      <c r="P7" s="65"/>
+      <c r="Q7" s="51" t="s">
         <v>58</v>
       </c>
-      <c r="R7" s="82"/>
-      <c r="S7" s="83"/>
-      <c r="T7" s="84"/>
-      <c r="U7" s="85"/>
-      <c r="V7" s="83"/>
-      <c r="W7" s="84"/>
-      <c r="X7" s="84"/>
-      <c r="Y7" s="86" t="s">
+      <c r="R7" s="66"/>
+      <c r="S7" s="67"/>
+      <c r="T7" s="61"/>
+      <c r="U7" s="68"/>
+      <c r="V7" s="67"/>
+      <c r="W7" s="61"/>
+      <c r="X7" s="61"/>
+      <c r="Y7" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="Z7" s="84"/>
-      <c r="AA7" s="84"/>
-      <c r="AB7" s="85"/>
-      <c r="AC7" s="87"/>
+      <c r="Z7" s="61"/>
+      <c r="AA7" s="61"/>
+      <c r="AB7" s="68"/>
+      <c r="AC7" s="69"/>
     </row>
     <row r="8" spans="1:29">
-      <c r="A8" s="88"/>
-      <c r="B8" s="89" t="s">
+      <c r="A8" s="70"/>
+      <c r="B8" s="70" t="s">
         <v>60</v>
       </c>
-      <c r="C8" s="89" t="s">
+      <c r="C8" s="70" t="s">
         <v>60</v>
       </c>
       <c r="D8" s="5">
         <v>0</v>
       </c>
-      <c r="E8" s="89" t="s">
+      <c r="E8" s="70" t="s">
         <v>61</v>
       </c>
       <c r="F8" s="5">
@@ -2059,11 +1978,6 @@
       <c r="G8" s="6">
         <v>0</v>
       </c>
-      <c r="H8" s="7"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="7"/>
       <c r="M8" s="8">
         <v>0</v>
       </c>
@@ -2082,19 +1996,18 @@
       <c r="R8" s="6">
         <v>0</v>
       </c>
-      <c r="S8" s="7"/>
-      <c r="AC8" s="90"/>
+      <c r="AC8" s="71"/>
     </row>
     <row r="9" spans="1:29">
-      <c r="A9" s="88"/>
-      <c r="B9" s="88"/>
-      <c r="C9" s="89" t="s">
+      <c r="A9" s="70"/>
+      <c r="B9" s="70"/>
+      <c r="C9" s="70" t="s">
         <v>60</v>
       </c>
       <c r="D9" s="5">
         <v>1</v>
       </c>
-      <c r="E9" s="89" t="s">
+      <c r="E9" s="70" t="s">
         <v>61</v>
       </c>
       <c r="F9" s="5">
@@ -2103,11 +2016,6 @@
       <c r="G9" s="6">
         <v>0</v>
       </c>
-      <c r="H9" s="7"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="7"/>
       <c r="M9" s="8">
         <v>0</v>
       </c>
@@ -2126,20 +2034,19 @@
       <c r="R9" s="6">
         <v>0</v>
       </c>
-      <c r="S9" s="7"/>
-      <c r="AC9" s="90"/>
+      <c r="AC9" s="71"/>
     </row>
     <row r="10" spans="1:29">
-      <c r="B10" s="91" t="s">
+      <c r="B10" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C10" s="91" t="s">
+      <c r="C10" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D10" s="5">
         <v>0</v>
       </c>
-      <c r="E10" s="91" t="s">
+      <c r="E10" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F10" s="5">
@@ -2148,7 +2055,7 @@
       <c r="G10" s="6">
         <v>0</v>
       </c>
-      <c r="H10" s="92" t="s">
+      <c r="H10" s="7" t="s">
         <v>64</v>
       </c>
       <c r="I10" s="5">
@@ -2162,13 +2069,13 @@
       </c>
     </row>
     <row r="11" spans="1:29">
-      <c r="C11" s="91" t="s">
+      <c r="C11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="5">
         <v>1</v>
       </c>
-      <c r="E11" s="91" t="s">
+      <c r="E11" s="5" t="s">
         <v>63</v>
       </c>
       <c r="F11" s="5">
@@ -2177,7 +2084,7 @@
       <c r="G11" s="6">
         <v>0</v>
       </c>
-      <c r="H11" s="92" t="s">
+      <c r="H11" s="7" t="s">
         <v>64</v>
       </c>
       <c r="I11" s="5">
@@ -2191,16 +2098,16 @@
       </c>
     </row>
     <row r="12" spans="1:29">
-      <c r="B12" s="91" t="s">
+      <c r="B12" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C12" s="91" t="s">
+      <c r="C12" s="5" t="s">
         <v>65</v>
       </c>
       <c r="D12" s="5">
         <v>0</v>
       </c>
-      <c r="E12" s="91" t="s">
+      <c r="E12" s="5" t="s">
         <v>66</v>
       </c>
       <c r="F12" s="5">
@@ -2218,7 +2125,6 @@
       <c r="O12" s="8">
         <v>0</v>
       </c>
-      <c r="P12" s="9"/>
       <c r="S12" s="7">
         <v>60</v>
       </c>
@@ -2229,7 +2135,7 @@
         <v>0</v>
       </c>
       <c r="V12" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W12" s="5">
         <v>0.1</v>
@@ -2237,10 +2143,10 @@
       <c r="X12" s="5">
         <v>5</v>
       </c>
-      <c r="Y12" s="91" t="s">
+      <c r="Y12" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="Z12" s="91" t="s">
+      <c r="Z12" s="5" t="s">
         <v>68</v>
       </c>
       <c r="AA12" s="5">
@@ -2251,13 +2157,13 @@
       </c>
     </row>
     <row r="13" spans="1:29">
-      <c r="C13" s="91" t="s">
+      <c r="C13" s="5" t="s">
         <v>65</v>
       </c>
       <c r="D13" s="5">
         <v>1</v>
       </c>
-      <c r="E13" s="91" t="s">
+      <c r="E13" s="5" t="s">
         <v>66</v>
       </c>
       <c r="F13" s="5">
@@ -2275,7 +2181,6 @@
       <c r="O13" s="8">
         <v>0</v>
       </c>
-      <c r="P13" s="9"/>
       <c r="S13" s="7">
         <v>60</v>
       </c>
@@ -2286,7 +2191,7 @@
         <v>0</v>
       </c>
       <c r="V13" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W13" s="5">
         <v>0.1</v>
@@ -2294,10 +2199,10 @@
       <c r="X13" s="5">
         <v>5</v>
       </c>
-      <c r="Y13" s="91" t="s">
+      <c r="Y13" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="Z13" s="91" t="s">
+      <c r="Z13" s="5" t="s">
         <v>68</v>
       </c>
       <c r="AA13" s="5">

</xml_diff>

<commit_message>
feat: Update equipment configurations and enhance combat mechanics
- Modified equip.xlsx and marble.xlsx files to reflect new equipment data.
- Increased maximum motor force for shield and sword prefabs to improve combat dynamics.
- Added spear configuration to gameplay_combat_tbequipment.json, enhancing weapon variety.
- Introduced lancer configuration in gameplay_combat_tbmarble.json, expanding character options.
- Adjusted Test.unity scene settings for better gameplay balance and character spawn configurations.
- Implemented collision handling in Equipment.cs and SwordEquipment.cs to improve combat interactions.
- Enhanced WeaponEquipment.cs to manage damage colliders, refining damage mechanics.
- Updated EquipmentMountAbility.cs to utilize AnchoredJoint2D for improved equipment attachment logic.
- Refactored SwordCollisionAttackAbility.cs to incorporate collider checks for damage handling.
</commit_message>
<xml_diff>
--- a/Configs/GameConfig/Datas/equip.xlsx
+++ b/Configs/GameConfig/Datas/equip.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="71">
   <si>
     <t>##var</t>
   </si>
@@ -239,6 +239,12 @@
   </si>
   <si>
     <t>arrow</t>
+  </si>
+  <si>
+    <t>spear</t>
+  </si>
+  <si>
+    <t>枪</t>
   </si>
 </sst>
 </file>
@@ -1517,7 +1523,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AC13"/>
+  <dimension ref="A1:AC14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9" style="5" customWidth="1"/>
@@ -2209,6 +2215,44 @@
         <v>0</v>
       </c>
       <c r="AB13" s="8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:29">
+      <c r="B14" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="D14" s="5">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="F14" s="5">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6">
+        <v>0</v>
+      </c>
+      <c r="M14" s="8">
+        <v>0</v>
+      </c>
+      <c r="N14" s="7">
+        <v>0.1</v>
+      </c>
+      <c r="O14" s="8">
+        <v>0</v>
+      </c>
+      <c r="P14" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="5">
+        <v>0.2</v>
+      </c>
+      <c r="R14" s="6">
         <v>0</v>
       </c>
     </row>

</xml_diff>